<commit_message>
Xlnt update; Script and window for update constrs data by db; DB data storage singleton
</commit_message>
<xml_diff>
--- a/assets/constructions/examples/ctd_arb_bush.xlsx
+++ b/assets/constructions/examples/ctd_arb_bush.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ctd" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ctd" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,47 +534,61 @@
           <t>releasepack</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>lcs</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>pricevalue</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>pricecurrency</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>pricevalue_rub</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SL4020</t>
+          <t>DBJ16-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LIKON</t>
+          <t>DEREK</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="n">
-        <v>71</v>
-      </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
+      <c r="D2" t="n">
+        <v>38</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>HB-20</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>HB-20</t>
+          <t>ISO_5609:12</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>LIKON</t>
+          <t>DEREK</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="L2" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="M2" t="n">
         <v>1</v>
@@ -585,7 +599,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>ZYL-40WIN</t>
+          <t>ZYL-16</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -596,14 +610,28 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2022/LIKON Инструментальный каталог</t>
-        </is>
+          <t>2019/DEREK Металлорежущий инструмент и оснастка</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W2" t="n">
+        <v>57.94</v>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y2" t="n">
+        <v>4749.57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DBJ12-8</t>
+          <t>CSO40-25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -611,17 +639,27 @@
           <t>DEREK</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Переходные втулки CSO к патронам с устройством для подачи СОЖ</t>
+        </is>
+      </c>
       <c r="D3" t="n">
-        <v>32</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+        <v>75</v>
+      </c>
+      <c r="E3" t="n">
+        <v>65</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>63</v>
+      </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ISO_5609:8</t>
+          <t>HB-25</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -630,10 +668,10 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="L3" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="M3" t="n">
         <v>1</v>
@@ -644,12 +682,14 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>ZYL-12</t>
+          <t>DER_SLO:HB-40</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>0.59</v>
+      </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
@@ -657,48 +697,56 @@
         <is>
           <t>2019/DEREK Металлорежущий инструмент и оснастка</t>
         </is>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W3" t="n">
+        <v>73.87</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y3" t="n">
+        <v>6055.41</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SL3225</t>
+          <t>DBJ12-8</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LIKON</t>
+          <t>DEREK</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="n">
-        <v>56</v>
-      </c>
-      <c r="F4" t="b">
-        <v>0</v>
-      </c>
+      <c r="D4" t="n">
+        <v>32</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>HB-25</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>HB-25</t>
+          <t>ISO_5609:8</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>LIKON</t>
+          <t>DEREK</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="L4" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="M4" t="n">
         <v>1</v>
@@ -709,7 +757,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>ZYL-32WIN</t>
+          <t>ZYL-12</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -720,54 +768,64 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2022/LIKON Инструментальный каталог</t>
-        </is>
+          <t>2019/DEREK Металлорежущий инструмент и оснастка</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W4" t="n">
+        <v>57.94</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y4" t="n">
+        <v>4749.57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CSO32-16</t>
+          <t>SL4008</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DEREK</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Переходные втулки CSO к патронам с устройством для подачи СОЖ</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>65</v>
-      </c>
+          <t>LIKON</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
-      <c r="G5" t="n">
-        <v>53</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>HB-8</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>HB-16</t>
+          <t>HB-8</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>DEREK</t>
+          <t>LIKON</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="L5" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M5" t="n">
         <v>1</v>
@@ -778,27 +836,35 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>DER_SLO:HB-32</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+          <t>ZYL-40</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr"/>
-      <c r="S5" t="n">
-        <v>0.4</v>
-      </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>0</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2019/DEREK Металлорежущий инструмент и оснастка</t>
-        </is>
-      </c>
+          <t>2022/LIKON Инструментальный каталог</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>1</v>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DBJ12-10</t>
+          <t>DBJ10-8</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -808,7 +874,7 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
@@ -816,7 +882,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ISO_5609:10</t>
+          <t>ISO_5609:8</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -825,10 +891,10 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L6" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M6" t="n">
         <v>1</v>
@@ -839,7 +905,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>ZYL-12</t>
+          <t>ZYL-10</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -853,6 +919,20 @@
           <t>2019/DEREK Металлорежущий инструмент и оснастка</t>
         </is>
       </c>
+      <c r="V6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" t="n">
+        <v>57.94</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>4749.57</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>